<commit_message>
v10: new 44-page report (Part A pipeline concepts, Part B advanced work, back matter) from program captures, plots of the code's formulas and the workbook; capture harness, figure / number / table generators, v10 benchmark set with CSV (p95), 2-minute showcase render log; old report moved to report/legacy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/workbooks/cg_workbook.xlsx
+++ b/report/workbooks/cg_workbook.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Ray_Tracing'!$A$1:$J$39</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Thermal_Kernels'!$A$1:$Z$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'Duty_Cycle'!$A$1:$Z$34</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'Performance'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'Performance'!$A$1:$I$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -363,6 +363,155 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Frame time per configuration (ms)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Performance'!B6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Performance'!$A$7:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Performance'!$B$7:$B$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Performance'!C6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Performance'!$A$7:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Performance'!$C$7:$C$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>ms</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3528,7 +3677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3620,54 +3769,382 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>TODO: no bench.csv yet</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>EPIC day 10:30</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>14.8698</v>
+      </c>
+      <c r="C7" s="24" t="n">
+        <v>17.7085</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>67.2503</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>256.151</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>5725520</v>
+      </c>
+      <c r="G7" s="27">
+        <f>IF(B7&gt;0,1000/B7,0)</f>
+        <v/>
+      </c>
+      <c r="H7" s="27">
+        <f>G7-D7</f>
+        <v/>
+      </c>
+      <c r="I7" s="7">
+        <f>IF(E7&gt;0,F7/E7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>EPIC night 23:00 (game: waves, UAVs)</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>16.3802</v>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>20.815</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>61.0493</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>970.4299999999999</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>5798500</v>
+      </c>
+      <c r="G8" s="27">
+        <f>IF(B8&gt;0,1000/B8,0)</f>
+        <v/>
+      </c>
+      <c r="H8" s="27">
+        <f>G8-D8</f>
+        <v/>
+      </c>
+      <c r="I8" s="7">
+        <f>IF(E8&gt;0,F8/E8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>EPIC day, thermal view</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>10.717</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>14.7982</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>93.30970000000001</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>71.2342</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>2726600</v>
+      </c>
+      <c r="G9" s="27">
+        <f>IF(B9&gt;0,1000/B9,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="27">
+        <f>G9-D9</f>
+        <v/>
+      </c>
+      <c r="I9" s="7">
+        <f>IF(E9&gt;0,F9/E9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>EPIC night, thermal view</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>12.6203</v>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>17.6151</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>79.2376</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>66.98399999999999</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>2499130</v>
+      </c>
+      <c r="G10" s="27">
+        <f>IF(B10&gt;0,1000/B10,0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="27">
+        <f>G10-D10</f>
+        <v/>
+      </c>
+      <c r="I10" s="7">
+        <f>IF(E10&gt;0,F10/E10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>EPIC day, shadows off</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>16.4236</v>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>21.0203</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>60.8879</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>205.716</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>5857520</v>
+      </c>
+      <c r="G11" s="27">
+        <f>IF(B11&gt;0,1000/B11,0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="27">
+        <f>G11-D11</f>
+        <v/>
+      </c>
+      <c r="I11" s="7">
+        <f>IF(E11&gt;0,F11/E11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>EPIC night, shadows off</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>17.1765</v>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>22.0255</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>58.2192</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>905.495</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>5867990</v>
+      </c>
+      <c r="G12" s="27">
+        <f>IF(B12&gt;0,1000/B12,0)</f>
+        <v/>
+      </c>
+      <c r="H12" s="27">
+        <f>G12-D12</f>
+        <v/>
+      </c>
+      <c r="I12" s="7">
+        <f>IF(E12&gt;0,F12/E12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>EPIC day, non-indexed</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>54.4709</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>59.4733</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>18.3584</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>4045.85</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>5855790</v>
+      </c>
+      <c r="G13" s="27">
+        <f>IF(B13&gt;0,1000/B13,0)</f>
+        <v/>
+      </c>
+      <c r="H13" s="27">
+        <f>G13-D13</f>
+        <v/>
+      </c>
+      <c r="I13" s="7">
+        <f>IF(E13&gt;0,F13/E13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>ULTRA day</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>16.7587</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>22.0811</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>59.6704</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>257.236</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>4307730</v>
+      </c>
+      <c r="G14" s="27">
+        <f>IF(B14&gt;0,1000/B14,0)</f>
+        <v/>
+      </c>
+      <c r="H14" s="27">
+        <f>G14-D14</f>
+        <v/>
+      </c>
+      <c r="I14" s="7">
+        <f>IF(E14&gt;0,F14/E14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>HIGH day</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>15.1059</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>17.2516</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>66.1991</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>168.717</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>1411360</v>
+      </c>
+      <c r="G15" s="27">
+        <f>IF(B15&gt;0,1000/B15,0)</f>
+        <v/>
+      </c>
+      <c r="H15" s="27">
+        <f>G15-D15</f>
+        <v/>
+      </c>
+      <c r="I15" s="7">
+        <f>IF(E15&gt;0,F15/E15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>LOW day</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>14.1625</v>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>16.0442</v>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>70.60899999999999</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>165.434</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>1315170</v>
+      </c>
+      <c r="G16" s="27">
+        <f>IF(B16&gt;0,1000/B16,0)</f>
+        <v/>
+      </c>
+      <c r="H16" s="27">
+        <f>G16-D16</f>
+        <v/>
+      </c>
+      <c r="I16" s="7">
+        <f>IF(E16&gt;0,F16/E16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>v1 look (no post) day</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="n">
+        <v>13.009</v>
+      </c>
+      <c r="C17" s="24" t="n">
+        <v>14.6926</v>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>76.87</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>148</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>1341050</v>
+      </c>
+      <c r="G17" s="27">
+        <f>IF(B17&gt;0,1000/B17,0)</f>
+        <v/>
+      </c>
+      <c r="H17" s="27">
+        <f>G17-D17</f>
+        <v/>
+      </c>
+      <c r="I17" s="7">
+        <f>IF(E17&gt;0,F17/E17,0)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <printOptions gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
report M1: legible figures (workbook blocks typeset + vector workbook appendix, plot layouts, state / architecture diagrams, banner, Frame Explorer insets, shading tiles)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/workbooks/cg_workbook.xlsx
+++ b/report/workbooks/cg_workbook.xlsx
@@ -4152,7 +4152,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:T202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -15960,7 +15960,7 @@
   </sheetData>
   <printOptions gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="75"/>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="41" min="0" max="16383" man="1"/>
     <brk id="124" min="0" max="16383" man="1"/>
@@ -20662,7 +20662,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -22313,7 +22313,7 @@
   </sheetData>
   <printOptions gridLines="0"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="78"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
report round 6 (bunker update): export at d99baa9 (Command bunker 403 parts, scene 5489), hinged blast gate in the card, chains, worked example and dynamics section; two searchlight shafts; workbook rebuilt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/workbooks/cg_workbook.xlsx
+++ b/report/workbooks/cg_workbook.xlsx
@@ -1183,7 +1183,7 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>2443</v>
+        <v>2452</v>
       </c>
       <c r="Q7" s="7">
         <f>M7*P7</f>
@@ -1252,7 +1252,7 @@
         <v/>
       </c>
       <c r="P8" s="8" t="n">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="Q8" s="7">
         <f>M8*P8</f>
@@ -1392,7 +1392,7 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="Q10" s="7">
         <f>M10*P10</f>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
@@ -11036,7 +11036,7 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="8" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>1</v>
@@ -11045,7 +11045,7 @@
         <v>9</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
@@ -11058,7 +11058,7 @@
         <v/>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>427</v>
+        <v>440</v>
       </c>
       <c r="R10" s="15">
         <f>IF(P10=Q10,"OK","DIFF")</f>
@@ -12736,7 +12736,7 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>2467</v>
+        <v>2476</v>
       </c>
       <c r="C39" s="8" t="n">
         <v>6</v>
@@ -12748,7 +12748,7 @@
         <v>2</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="G39" s="8" t="n">
         <v>10</v>
@@ -12757,7 +12757,7 @@
         <v>364</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="J39" s="8" t="n">
         <v>3</v>
@@ -12782,7 +12782,7 @@
         <v/>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>5476</v>
+        <v>5489</v>
       </c>
     </row>
     <row r="40">
@@ -23846,10 +23846,10 @@
         <v>1</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>390</v>
+        <v>403</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>390</v>
+        <v>403</v>
       </c>
       <c r="F20" s="7">
         <f>IF(ISNUMBER(D20),C20*D20,E20)</f>
@@ -23857,7 +23857,7 @@
       </c>
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="8" t="n">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="I20" s="8" t="n">
         <v>1</v>
@@ -23865,7 +23865,7 @@
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="8" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="M20" s="8" t="n">
         <v>1</v>
@@ -23874,7 +23874,7 @@
         <v>9</v>
       </c>
       <c r="O20" s="8" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
@@ -26515,7 +26515,7 @@
         </is>
       </c>
       <c r="E70" s="8" t="n">
-        <v>5476</v>
+        <v>5489</v>
       </c>
       <c r="F70" s="15">
         <f>IF(E69=E70,"OK","DIFF")</f>
@@ -32913,7 +32913,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: scene/DayCycle (solar model, transmittance, 3.2 smoothstep(-1, 10, e), ambient mixLog); export 'lights'; ShaderSources.cpp brdf(); BNK-171 'Roof slab A'.</t>
+          <t>Source: scene/DayCycle (solar model, transmittance, 3.2 smoothstep(-1, 10, e), ambient mixLog); export 'lights'; ShaderSources.cpp brdf(); the command bunker's part 'Roof slab A'.</t>
         </is>
       </c>
     </row>
@@ -33510,7 +33510,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>roof albedo kd (BNK-171 colour)</t>
+          <t>roof albedo kd (Roof slab A colour)</t>
         </is>
       </c>
       <c r="I19" s="16" t="n">

</xml_diff>

<commit_message>
final night (part 3): 3:38 film assembler (gen_film3.py) and recorder camera steps; report on the final export (5,474 parts): hand-written vector maths subsection, coordinate sheet per design in Section 7, full forms in every title, flow diagrams as one-row chains, whole-base motion figures, single / combined strike, guards, alert posture and boarding described
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/workbooks/cg_workbook.xlsx
+++ b/report/workbooks/cg_workbook.xlsx
@@ -1183,7 +1183,7 @@
         <v/>
       </c>
       <c r="P7" s="8" t="n">
-        <v>2452</v>
+        <v>2453</v>
       </c>
       <c r="Q7" s="7">
         <f>M7*P7</f>
@@ -1392,7 +1392,7 @@
         <v/>
       </c>
       <c r="P10" s="8" t="n">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="Q10" s="7">
         <f>M10*P10</f>
@@ -1891,7 +1891,7 @@
         <v/>
       </c>
       <c r="P17" s="8" t="n">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="Q17" s="7">
         <f>M17*P17</f>
@@ -10881,7 +10881,9 @@
           <t>Backdrop</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
+      <c r="B8" s="8" t="n">
+        <v>4</v>
+      </c>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
@@ -10891,7 +10893,7 @@
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="8" t="n">
@@ -10906,7 +10908,7 @@
         <v/>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="R8" s="15">
         <f>IF(P8=Q8,"OK","DIFF")</f>
@@ -12055,7 +12057,7 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
@@ -12065,7 +12067,7 @@
       </c>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="8" t="n">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="I25" s="8" t="n">
         <v>90</v>
@@ -12083,7 +12085,7 @@
         <v/>
       </c>
       <c r="Q25" s="8" t="n">
-        <v>658</v>
+        <v>640</v>
       </c>
       <c r="R25" s="15">
         <f>IF(P25=Q25,"OK","DIFF")</f>
@@ -12736,7 +12738,7 @@
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>2476</v>
+        <v>2477</v>
       </c>
       <c r="C39" s="8" t="n">
         <v>6</v>
@@ -12754,10 +12756,10 @@
         <v>10</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="J39" s="8" t="n">
         <v>3</v>
@@ -12782,7 +12784,7 @@
         <v/>
       </c>
       <c r="Q39" s="8" t="n">
-        <v>5489</v>
+        <v>5474</v>
       </c>
     </row>
     <row r="40">
@@ -24937,11 +24939,11 @@
       </c>
       <c r="D40" s="18" t="inlineStr">
         <is>
-          <t>48..60</t>
+          <t>42..56</t>
         </is>
       </c>
       <c r="E40" s="8" t="n">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="F40" s="7">
         <f>IF(ISNUMBER(D40),C40*D40,E40)</f>
@@ -24949,7 +24951,7 @@
       </c>
       <c r="G40" s="7" t="n"/>
       <c r="H40" s="8" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="7" t="n"/>
@@ -24957,7 +24959,7 @@
       <c r="L40" s="7" t="n"/>
       <c r="M40" s="7" t="n"/>
       <c r="N40" s="8" t="n">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="O40" s="7" t="n"/>
       <c r="P40" s="7" t="n"/>
@@ -26135,29 +26137,29 @@
         </is>
       </c>
       <c r="C63" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D63" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F63" s="7">
         <f>IF(ISNUMBER(D63),C63*D63,E63)</f>
         <v/>
       </c>
       <c r="G63" s="7" t="n"/>
-      <c r="H63" s="7" t="n"/>
+      <c r="H63" s="8" t="n">
+        <v>4</v>
+      </c>
       <c r="I63" s="7" t="n"/>
       <c r="J63" s="7" t="n"/>
       <c r="K63" s="7" t="n"/>
       <c r="L63" s="7" t="n"/>
       <c r="M63" s="7" t="n"/>
       <c r="N63" s="7" t="n"/>
-      <c r="O63" s="8" t="n">
-        <v>1</v>
-      </c>
+      <c r="O63" s="7" t="n"/>
       <c r="P63" s="7" t="n"/>
       <c r="Q63" s="7" t="n"/>
       <c r="R63" s="7" t="n"/>
@@ -26515,7 +26517,7 @@
         </is>
       </c>
       <c r="E70" s="8" t="n">
-        <v>5489</v>
+        <v>5474</v>
       </c>
       <c r="F70" s="15">
         <f>IF(E69=E70,"OK","DIFF")</f>

</xml_diff>